<commit_message>
feat: agregar CONCEPTO al pipeline efectivo y 5_cobranza (DE7-CODE)
- 4_pagos/efectivo: leer_hoja() lee CONCEPTO, exportar escribe badges de color
- crear_templates.py: CONCEPTO incluido en mesa template futuro
- mesa_5/mesa_6: columna CONCEPTO agregada sin perder datos
- 5_cobranza: loaders leen concepto, calcular filtra agua, trazabilidad col 7
- 5_cobranza: --force flag para recalcular sin pagos nuevos
- A-3 mesa_6 corregido: S/200 tanque separado del agua
- EXCESO 17->13, CANCELADO 291->295 tras correcciones CORTE_RECONEXION

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/inputs/mesa_6.xlsx
+++ b/4_pagos/efectivo/inputs/mesa_6.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilde\PycharmProjects\jass_system\4_pagos\efectivo\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEADA9AE-31CC-481B-8DB6-1BE022A11807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862580BE-1E3C-4BB4-B7FB-5734BBC91EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-27660" yWindow="0" windowWidth="14610" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="registro_1" sheetId="1" r:id="rId1"/>
     <sheet name="registro_2" sheetId="2" r:id="rId2"/>
     <sheet name="registro_3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">registro_1!$A$2:$K$80</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="69">
   <si>
     <t>¿Quién cobró?</t>
   </si>
@@ -50,6 +53,9 @@
     <t>¿Alguna nota?</t>
   </si>
   <si>
+    <t>¿Qué tipo?</t>
+  </si>
+  <si>
     <t>COBRADOR</t>
   </si>
   <si>
@@ -77,6 +83,9 @@
     <t>COMENTARIO</t>
   </si>
   <si>
+    <t>CONCEPTO</t>
+  </si>
+  <si>
     <t>María García</t>
   </si>
   <si>
@@ -101,24 +110,42 @@
     <t>03/06/2026</t>
   </si>
   <si>
+    <t>tanque</t>
+  </si>
+  <si>
     <t>Wagner Trujillo</t>
   </si>
   <si>
     <t>P</t>
   </si>
   <si>
+    <t>compromiso + exoneracion</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
     <t>G</t>
   </si>
   <si>
+    <t>BLANCO</t>
+  </si>
+  <si>
+    <t>Hernestina Valladares?</t>
+  </si>
+  <si>
     <t>Q</t>
   </si>
   <si>
     <t>60?</t>
   </si>
   <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t>Ocaña?</t>
+  </si>
+  <si>
     <t>16A</t>
   </si>
   <si>
@@ -128,6 +155,9 @@
     <t>Y</t>
   </si>
   <si>
+    <t>reclamo</t>
+  </si>
+  <si>
     <t>B1</t>
   </si>
   <si>
@@ -140,6 +170,9 @@
     <t>27A</t>
   </si>
   <si>
+    <t>K</t>
+  </si>
+  <si>
     <t>T</t>
   </si>
   <si>
@@ -155,6 +188,12 @@
     <t>C</t>
   </si>
   <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
@@ -170,18 +209,12 @@
     <t>U</t>
   </si>
   <si>
-    <t>reclamo</t>
-  </si>
-  <si>
-    <t>K</t>
+    <t>compromiso</t>
   </si>
   <si>
     <t>J</t>
   </si>
   <si>
-    <t>consumo +200 tanque</t>
-  </si>
-  <si>
     <t>F1</t>
   </si>
   <si>
@@ -194,6 +227,9 @@
     <t>G1</t>
   </si>
   <si>
+    <t>pago yape</t>
+  </si>
+  <si>
     <t>E</t>
   </si>
   <si>
@@ -203,47 +239,20 @@
     <t>C1</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>Hernestina Valladares?</t>
-  </si>
-  <si>
-    <t>Ocaña?</t>
-  </si>
-  <si>
-    <t>pago yape</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
     <t>V</t>
   </si>
   <si>
-    <t>H1</t>
+    <t>exonerado</t>
   </si>
   <si>
     <t>Z</t>
-  </si>
-  <si>
-    <t>exonerado</t>
-  </si>
-  <si>
-    <t>BLANCO</t>
-  </si>
-  <si>
-    <t>compromiso</t>
-  </si>
-  <si>
-    <t>compromiso + exoneracion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -305,8 +314,26 @@
       <color rgb="FF9CA3AF"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF9A3412"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF9A3412"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF9CA3AF"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -339,8 +366,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7ED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -348,11 +380,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -372,11 +419,18 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -689,102 +743,113 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K80"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.81640625" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="16" style="9" customWidth="1"/>
+    <col min="3" max="4" width="8" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12" style="9" customWidth="1"/>
+    <col min="6" max="6" width="16" style="9" customWidth="1"/>
+    <col min="7" max="8" width="14" style="9" customWidth="1"/>
+    <col min="9" max="9" width="30" style="9" customWidth="1"/>
+    <col min="10" max="10" width="14" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="12" t="s">
+    <row r="1" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="15" t="s">
+      <c r="D1" s="14"/>
+      <c r="E1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J1" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I3" s="6"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J3" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="8">
+        <v>24</v>
+      </c>
+      <c r="B4" s="7">
         <v>46181</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D4">
         <v>13</v>
@@ -792,28 +857,28 @@
       <c r="E4">
         <v>36</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4">
         <v>36</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <v>46178</v>
       </c>
       <c r="I4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="8">
+        <v>24</v>
+      </c>
+      <c r="B5" s="7">
         <v>46181</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -821,25 +886,25 @@
       <c r="E5">
         <v>34</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5">
         <v>34</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="8">
+        <v>24</v>
+      </c>
+      <c r="B6" s="7">
         <v>46181</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D6">
         <v>12</v>
@@ -847,51 +912,51 @@
       <c r="E6">
         <v>34</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6">
         <v>34</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="8">
+        <v>24</v>
+      </c>
+      <c r="B7" s="7">
         <v>46181</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E7">
         <v>45</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7">
         <v>45</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="7">
         <v>46178</v>
       </c>
       <c r="I7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="8">
+        <v>24</v>
+      </c>
+      <c r="B8" s="7">
         <v>46181</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -899,28 +964,28 @@
       <c r="E8">
         <v>60</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8">
         <v>60</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="7">
         <v>46178</v>
       </c>
       <c r="I8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="8">
+        <v>24</v>
+      </c>
+      <c r="B9" s="7">
         <v>46181</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -928,54 +993,54 @@
       <c r="E9">
         <v>80</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9">
         <v>80</v>
       </c>
-      <c r="G9" s="10">
-        <v>0</v>
-      </c>
-      <c r="H9" s="8">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7">
         <v>46178</v>
       </c>
       <c r="I9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="8">
+        <v>24</v>
+      </c>
+      <c r="B10" s="7">
         <v>46181</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E10">
         <v>25</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10">
         <v>25</v>
       </c>
-      <c r="G10" s="10">
-        <v>0</v>
-      </c>
-      <c r="H10" s="8">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="8">
+        <v>24</v>
+      </c>
+      <c r="B11" s="7">
         <v>46181</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D11">
         <v>11</v>
@@ -983,25 +1048,25 @@
       <c r="E11">
         <v>33</v>
       </c>
-      <c r="F11" s="7">
+      <c r="F11">
         <v>33</v>
       </c>
-      <c r="G11" s="10">
-        <v>0</v>
-      </c>
-      <c r="H11" s="8">
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="8">
+        <v>24</v>
+      </c>
+      <c r="B12" s="7">
         <v>46181</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D12">
         <v>6</v>
@@ -1009,28 +1074,28 @@
       <c r="E12">
         <v>102</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F12">
         <v>102</v>
       </c>
-      <c r="G12" s="10">
-        <v>0</v>
-      </c>
-      <c r="H12" s="8">
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12" s="7">
         <v>46178</v>
       </c>
       <c r="I12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="8">
+        <v>24</v>
+      </c>
+      <c r="B13" s="7">
         <v>46181</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1038,25 +1103,25 @@
       <c r="E13">
         <v>71</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13">
         <v>71</v>
       </c>
-      <c r="G13" s="10">
-        <v>0</v>
-      </c>
-      <c r="H13" s="8">
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="8">
+        <v>24</v>
+      </c>
+      <c r="B14" s="7">
         <v>46181</v>
       </c>
       <c r="C14" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1064,25 +1129,25 @@
       <c r="E14">
         <v>50</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14">
         <v>50</v>
       </c>
-      <c r="G14" s="10">
-        <v>0</v>
-      </c>
-      <c r="H14" s="8">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="8">
+        <v>24</v>
+      </c>
+      <c r="B15" s="7">
         <v>46181</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1090,54 +1155,54 @@
       <c r="E15">
         <v>20</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15">
         <v>20</v>
       </c>
-      <c r="G15" s="10">
-        <v>0</v>
-      </c>
-      <c r="H15" s="8">
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" s="7">
         <v>46178</v>
       </c>
       <c r="I15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="8">
+        <v>24</v>
+      </c>
+      <c r="B16" s="7">
         <v>46181</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E16">
         <v>28</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16">
         <v>28</v>
       </c>
-      <c r="G16" s="10">
-        <v>0</v>
-      </c>
-      <c r="H16" s="8">
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="8">
+        <v>24</v>
+      </c>
+      <c r="B17" s="7">
         <v>46181</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D17">
         <v>9</v>
@@ -1145,28 +1210,28 @@
       <c r="E17">
         <v>0</v>
       </c>
-      <c r="F17" s="7">
-        <v>0</v>
-      </c>
-      <c r="G17" s="10">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8">
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" s="7">
         <v>46178</v>
       </c>
       <c r="I17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C18" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="8">
-        <v>46181</v>
-      </c>
-      <c r="C18" t="s">
-        <v>34</v>
       </c>
       <c r="D18">
         <v>12</v>
@@ -1174,25 +1239,25 @@
       <c r="E18">
         <v>155</v>
       </c>
-      <c r="F18" s="7">
+      <c r="F18">
         <v>0</v>
       </c>
       <c r="G18">
         <v>155</v>
       </c>
-      <c r="H18" s="8">
+      <c r="H18" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="8">
+        <v>24</v>
+      </c>
+      <c r="B19" s="7">
         <v>46181</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D19">
         <v>15</v>
@@ -1200,25 +1265,25 @@
       <c r="E19">
         <v>38</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19">
         <v>38</v>
       </c>
       <c r="G19">
         <v>0</v>
       </c>
-      <c r="H19" s="8">
+      <c r="H19" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="8">
+        <v>24</v>
+      </c>
+      <c r="B20" s="7">
         <v>46181</v>
       </c>
       <c r="C20" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -1226,25 +1291,25 @@
       <c r="E20">
         <v>58</v>
       </c>
-      <c r="F20" s="7">
+      <c r="F20">
         <v>58</v>
       </c>
       <c r="G20">
         <v>0</v>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="8">
+        <v>24</v>
+      </c>
+      <c r="B21" s="7">
         <v>46181</v>
       </c>
       <c r="C21" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D21">
         <v>6</v>
@@ -1252,25 +1317,25 @@
       <c r="E21">
         <v>53</v>
       </c>
-      <c r="F21" s="7">
+      <c r="F21">
         <v>53</v>
       </c>
-      <c r="G21" s="10">
-        <v>0</v>
-      </c>
-      <c r="H21" s="8">
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="8">
+        <v>24</v>
+      </c>
+      <c r="B22" s="7">
         <v>46181</v>
       </c>
       <c r="C22" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D22">
         <v>18</v>
@@ -1278,25 +1343,25 @@
       <c r="E22">
         <v>36</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22">
         <v>36</v>
       </c>
-      <c r="G22" s="10">
-        <v>0</v>
-      </c>
-      <c r="H22" s="8">
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="8">
+        <v>24</v>
+      </c>
+      <c r="B23" s="7">
         <v>46181</v>
       </c>
       <c r="C23" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D23">
         <v>20</v>
@@ -1304,25 +1369,25 @@
       <c r="E23">
         <v>110</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23">
         <v>110</v>
       </c>
-      <c r="G23" s="10">
-        <v>0</v>
-      </c>
-      <c r="H23" s="8">
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="8">
+        <v>24</v>
+      </c>
+      <c r="B24" s="7">
         <v>46181</v>
       </c>
       <c r="C24" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D24">
         <v>4</v>
@@ -1330,25 +1395,25 @@
       <c r="E24">
         <v>28</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24">
         <v>28</v>
       </c>
-      <c r="G24" s="10">
-        <v>0</v>
-      </c>
-      <c r="H24" s="8">
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="8">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7">
         <v>46181</v>
       </c>
       <c r="C25" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D25">
         <v>12</v>
@@ -1356,25 +1421,25 @@
       <c r="E25">
         <v>15</v>
       </c>
-      <c r="F25" s="7">
+      <c r="F25">
         <v>15</v>
       </c>
-      <c r="G25" s="10">
-        <v>0</v>
-      </c>
-      <c r="H25" s="8">
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>21</v>
-      </c>
-      <c r="B26" s="8">
+        <v>24</v>
+      </c>
+      <c r="B26" s="7">
         <v>46181</v>
       </c>
       <c r="C26" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D26">
         <v>16</v>
@@ -1382,25 +1447,25 @@
       <c r="E26">
         <v>33</v>
       </c>
-      <c r="F26" s="7">
+      <c r="F26">
         <v>33</v>
       </c>
-      <c r="G26" s="10">
-        <v>0</v>
-      </c>
-      <c r="H26" s="8">
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="8">
+        <v>24</v>
+      </c>
+      <c r="B27" s="7">
         <v>46181</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D27">
         <v>5</v>
@@ -1408,25 +1473,25 @@
       <c r="E27">
         <v>8</v>
       </c>
-      <c r="F27" s="7">
+      <c r="F27">
         <v>8</v>
       </c>
-      <c r="G27" s="10">
-        <v>0</v>
-      </c>
-      <c r="H27" s="8">
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>21</v>
-      </c>
-      <c r="B28" s="8">
+        <v>24</v>
+      </c>
+      <c r="B28" s="7">
         <v>46181</v>
       </c>
       <c r="C28" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D28">
         <v>11</v>
@@ -1434,25 +1499,25 @@
       <c r="E28">
         <v>63</v>
       </c>
-      <c r="F28" s="7">
+      <c r="F28">
         <v>63</v>
       </c>
-      <c r="G28" s="10">
-        <v>0</v>
-      </c>
-      <c r="H28" s="8">
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>21</v>
-      </c>
-      <c r="B29" s="8">
+        <v>24</v>
+      </c>
+      <c r="B29" s="7">
         <v>46181</v>
       </c>
       <c r="C29" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="D29">
         <v>5</v>
@@ -1460,25 +1525,25 @@
       <c r="E29">
         <v>71</v>
       </c>
-      <c r="F29" s="7">
+      <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
         <v>71</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B30" s="8">
+        <v>24</v>
+      </c>
+      <c r="B30" s="7">
         <v>46181</v>
       </c>
       <c r="C30" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D30">
         <v>17</v>
@@ -1486,25 +1551,25 @@
       <c r="E30">
         <v>121</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30">
         <v>121</v>
       </c>
       <c r="G30">
         <v>0</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>21</v>
-      </c>
-      <c r="B31" s="8">
+        <v>24</v>
+      </c>
+      <c r="B31" s="7">
         <v>46181</v>
       </c>
       <c r="C31" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="D31">
         <v>16</v>
@@ -1512,25 +1577,25 @@
       <c r="E31">
         <v>85</v>
       </c>
-      <c r="F31" s="7">
+      <c r="F31">
         <v>0</v>
       </c>
       <c r="G31">
         <v>85</v>
       </c>
-      <c r="H31" s="8">
+      <c r="H31" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>21</v>
-      </c>
-      <c r="B32" s="8">
+        <v>24</v>
+      </c>
+      <c r="B32" s="7">
         <v>46181</v>
       </c>
       <c r="C32" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="D32">
         <v>6</v>
@@ -1538,25 +1603,25 @@
       <c r="E32">
         <v>33</v>
       </c>
-      <c r="F32" s="7">
+      <c r="F32">
         <v>0</v>
       </c>
       <c r="G32">
         <v>33</v>
       </c>
-      <c r="H32" s="8">
+      <c r="H32" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>21</v>
-      </c>
-      <c r="B33" s="8">
+        <v>24</v>
+      </c>
+      <c r="B33" s="7">
         <v>46181</v>
       </c>
       <c r="C33" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="D33">
         <v>9</v>
@@ -1564,25 +1629,25 @@
       <c r="E33">
         <v>86</v>
       </c>
-      <c r="F33" s="7">
+      <c r="F33">
         <v>0</v>
       </c>
       <c r="G33">
         <v>86</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>21</v>
-      </c>
-      <c r="B34" s="8">
+        <v>24</v>
+      </c>
+      <c r="B34" s="7">
         <v>46181</v>
       </c>
       <c r="C34" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -1590,25 +1655,25 @@
       <c r="E34">
         <v>58</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34">
         <v>0</v>
       </c>
       <c r="G34">
         <v>58</v>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="7">
         <v>46178</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>21</v>
-      </c>
-      <c r="B35" s="8">
+        <v>24</v>
+      </c>
+      <c r="B35" s="7">
         <v>46181</v>
       </c>
       <c r="C35" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D35">
         <v>2</v>
@@ -1616,33 +1681,33 @@
       <c r="E35">
         <v>25</v>
       </c>
-      <c r="F35" s="7">
+      <c r="F35">
         <v>25</v>
       </c>
       <c r="G35">
         <v>0</v>
       </c>
-      <c r="H35" s="8">
+      <c r="H35" s="7">
         <v>46178</v>
       </c>
-      <c r="J35" s="9">
+      <c r="J35" s="8">
         <f>SUM(F4:F35)</f>
         <v>1206</v>
       </c>
-      <c r="K35" s="9">
+      <c r="K35" s="8">
         <f>SUM(G4:G35)</f>
         <v>488</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>21</v>
-      </c>
-      <c r="B36" s="8">
+        <v>24</v>
+      </c>
+      <c r="B36" s="7">
         <v>46181</v>
       </c>
       <c r="C36" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="D36">
         <v>4</v>
@@ -1650,25 +1715,25 @@
       <c r="E36">
         <v>8</v>
       </c>
-      <c r="F36" s="7">
+      <c r="F36">
         <v>8</v>
       </c>
       <c r="G36">
         <v>0</v>
       </c>
-      <c r="H36" s="8">
+      <c r="H36" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>21</v>
-      </c>
-      <c r="B37" s="8">
+        <v>24</v>
+      </c>
+      <c r="B37" s="7">
         <v>46181</v>
       </c>
       <c r="C37" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D37">
         <v>15</v>
@@ -1676,25 +1741,28 @@
       <c r="E37">
         <v>100</v>
       </c>
-      <c r="F37" s="7">
+      <c r="F37">
         <v>100</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
-      <c r="H37" s="8">
+      <c r="H37" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I37" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>21</v>
-      </c>
-      <c r="B38" s="8">
+        <v>24</v>
+      </c>
+      <c r="B38" s="7">
         <v>46181</v>
       </c>
       <c r="C38" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D38">
         <v>6</v>
@@ -1702,25 +1770,25 @@
       <c r="E38">
         <v>383</v>
       </c>
-      <c r="F38" s="7">
+      <c r="F38">
         <v>383</v>
       </c>
-      <c r="G38" s="10">
-        <v>0</v>
-      </c>
-      <c r="H38" s="8">
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>21</v>
-      </c>
-      <c r="B39" s="8">
+        <v>24</v>
+      </c>
+      <c r="B39" s="7">
         <v>46181</v>
       </c>
       <c r="C39" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D39">
         <v>14</v>
@@ -1728,25 +1796,28 @@
       <c r="E39">
         <v>70</v>
       </c>
-      <c r="F39" s="7">
+      <c r="F39">
         <v>70</v>
       </c>
-      <c r="G39" s="10">
-        <v>0</v>
-      </c>
-      <c r="H39" s="8">
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I39" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>21</v>
-      </c>
-      <c r="B40" s="8">
+        <v>24</v>
+      </c>
+      <c r="B40" s="7">
         <v>46181</v>
       </c>
       <c r="C40" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="D40">
         <v>4</v>
@@ -1754,25 +1825,28 @@
       <c r="E40">
         <v>62</v>
       </c>
-      <c r="F40" s="7">
+      <c r="F40">
         <v>62</v>
       </c>
-      <c r="G40" s="10">
-        <v>0</v>
-      </c>
-      <c r="H40" s="8">
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I40" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>21</v>
-      </c>
-      <c r="B41" s="8">
+        <v>24</v>
+      </c>
+      <c r="B41" s="7">
         <v>46181</v>
       </c>
       <c r="C41" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D41">
         <v>26</v>
@@ -1780,28 +1854,28 @@
       <c r="E41">
         <v>58</v>
       </c>
-      <c r="F41" s="7">
+      <c r="F41">
         <v>58</v>
       </c>
-      <c r="G41" s="10">
-        <v>0</v>
-      </c>
-      <c r="H41" s="8">
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41" s="7">
         <v>46179</v>
       </c>
       <c r="I41" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>21</v>
-      </c>
-      <c r="B42" s="8">
+        <v>24</v>
+      </c>
+      <c r="B42" s="7">
         <v>46181</v>
       </c>
       <c r="C42" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D42">
         <v>27</v>
@@ -1809,54 +1883,51 @@
       <c r="E42">
         <v>49</v>
       </c>
-      <c r="F42" s="7">
+      <c r="F42">
         <v>49</v>
       </c>
-      <c r="G42" s="10">
-        <v>0</v>
-      </c>
-      <c r="H42" s="8">
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42" s="7">
         <v>46179</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>21</v>
-      </c>
-      <c r="B43" s="8">
+        <v>24</v>
+      </c>
+      <c r="B43" s="7">
         <v>46181</v>
       </c>
       <c r="C43" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D43">
         <v>3</v>
       </c>
       <c r="E43">
-        <v>208</v>
-      </c>
-      <c r="F43" s="7">
-        <v>208</v>
-      </c>
-      <c r="G43" s="10">
-        <v>0</v>
-      </c>
-      <c r="H43" s="8">
+        <v>8</v>
+      </c>
+      <c r="F43">
+        <v>8</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43" s="7">
         <v>46179</v>
       </c>
-      <c r="I43" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>21</v>
-      </c>
-      <c r="B44" s="8">
+        <v>24</v>
+      </c>
+      <c r="B44" s="7">
         <v>46181</v>
       </c>
       <c r="C44" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D44">
         <v>13</v>
@@ -1864,25 +1935,28 @@
       <c r="E44">
         <v>50</v>
       </c>
-      <c r="F44" s="7">
+      <c r="F44">
         <v>50</v>
       </c>
-      <c r="G44" s="10">
-        <v>0</v>
-      </c>
-      <c r="H44" s="8">
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I44" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>21</v>
-      </c>
-      <c r="B45" s="8">
+        <v>24</v>
+      </c>
+      <c r="B45" s="7">
         <v>46181</v>
       </c>
       <c r="C45" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="D45">
         <v>6</v>
@@ -1890,25 +1964,28 @@
       <c r="E45">
         <v>84</v>
       </c>
-      <c r="F45" s="7">
+      <c r="F45">
         <v>84</v>
       </c>
-      <c r="G45" s="10">
-        <v>0</v>
-      </c>
-      <c r="H45" s="8">
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I45" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>21</v>
-      </c>
-      <c r="B46" s="8">
+        <v>24</v>
+      </c>
+      <c r="B46" s="7">
         <v>46181</v>
       </c>
       <c r="C46" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D46">
         <v>19</v>
@@ -1916,25 +1993,25 @@
       <c r="E46">
         <v>85</v>
       </c>
-      <c r="F46" s="7">
+      <c r="F46">
         <v>85</v>
       </c>
-      <c r="G46" s="10">
-        <v>0</v>
-      </c>
-      <c r="H46" s="8">
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>21</v>
-      </c>
-      <c r="B47" s="8">
+        <v>24</v>
+      </c>
+      <c r="B47" s="7">
         <v>46181</v>
       </c>
       <c r="C47" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="D47">
         <v>12</v>
@@ -1942,25 +2019,25 @@
       <c r="E47">
         <v>116</v>
       </c>
-      <c r="F47" s="7">
+      <c r="F47">
         <v>116</v>
       </c>
-      <c r="G47" s="10">
-        <v>0</v>
-      </c>
-      <c r="H47" s="8">
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>21</v>
-      </c>
-      <c r="B48" s="8">
+        <v>24</v>
+      </c>
+      <c r="B48" s="7">
         <v>46181</v>
       </c>
       <c r="C48" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D48">
         <v>5</v>
@@ -1968,25 +2045,28 @@
       <c r="E48">
         <v>46</v>
       </c>
-      <c r="F48" s="7">
+      <c r="F48">
         <v>46</v>
       </c>
-      <c r="G48" s="10">
-        <v>0</v>
-      </c>
-      <c r="H48" s="8">
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I48" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>21</v>
-      </c>
-      <c r="B49" s="8">
+        <v>24</v>
+      </c>
+      <c r="B49" s="7">
         <v>46181</v>
       </c>
       <c r="C49" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D49">
         <v>1</v>
@@ -1994,25 +2074,28 @@
       <c r="E49">
         <v>62</v>
       </c>
-      <c r="F49" s="7">
+      <c r="F49">
         <v>62</v>
       </c>
-      <c r="G49" s="10">
-        <v>0</v>
-      </c>
-      <c r="H49" s="8">
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I49" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>21</v>
-      </c>
-      <c r="B50" s="8">
+        <v>24</v>
+      </c>
+      <c r="B50" s="7">
         <v>46181</v>
       </c>
       <c r="C50" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="D50">
         <v>11</v>
@@ -2020,28 +2103,28 @@
       <c r="E50">
         <v>50</v>
       </c>
-      <c r="F50" s="7">
+      <c r="F50">
         <v>50</v>
       </c>
-      <c r="G50" s="10">
-        <v>0</v>
-      </c>
-      <c r="H50" s="8">
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50" s="7">
         <v>46179</v>
       </c>
       <c r="I50" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>21</v>
-      </c>
-      <c r="B51" s="8">
+        <v>24</v>
+      </c>
+      <c r="B51" s="7">
         <v>46181</v>
       </c>
       <c r="C51" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="D51">
         <v>4</v>
@@ -2049,25 +2132,25 @@
       <c r="E51">
         <v>61</v>
       </c>
-      <c r="F51" s="7">
+      <c r="F51">
         <v>61</v>
       </c>
-      <c r="G51" s="10">
-        <v>0</v>
-      </c>
-      <c r="H51" s="8">
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>21</v>
-      </c>
-      <c r="B52" s="8">
+        <v>24</v>
+      </c>
+      <c r="B52" s="7">
         <v>46181</v>
       </c>
       <c r="C52" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D52">
         <v>5</v>
@@ -2075,25 +2158,28 @@
       <c r="E52">
         <v>14</v>
       </c>
-      <c r="F52" s="7">
+      <c r="F52">
         <v>14</v>
       </c>
-      <c r="G52" s="10">
-        <v>0</v>
-      </c>
-      <c r="H52" s="8">
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I52" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>21</v>
-      </c>
-      <c r="B53" s="8">
+        <v>24</v>
+      </c>
+      <c r="B53" s="7">
         <v>46181</v>
       </c>
       <c r="C53" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D53">
         <v>14</v>
@@ -2101,25 +2187,28 @@
       <c r="E53">
         <v>58</v>
       </c>
-      <c r="F53" s="7">
+      <c r="F53">
         <v>58</v>
       </c>
-      <c r="G53" s="10">
-        <v>0</v>
-      </c>
-      <c r="H53" s="8">
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I53" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>21</v>
-      </c>
-      <c r="B54" s="8">
+        <v>24</v>
+      </c>
+      <c r="B54" s="7">
         <v>46181</v>
       </c>
       <c r="C54" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="D54">
         <v>13</v>
@@ -2127,28 +2216,28 @@
       <c r="E54">
         <v>35</v>
       </c>
-      <c r="F54" s="7">
+      <c r="F54">
         <v>35</v>
       </c>
-      <c r="G54" s="10">
-        <v>0</v>
-      </c>
-      <c r="H54" s="8">
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54" s="7">
         <v>46179</v>
       </c>
       <c r="I54" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>21</v>
-      </c>
-      <c r="B55" s="8">
+        <v>24</v>
+      </c>
+      <c r="B55" s="7">
         <v>46181</v>
       </c>
       <c r="C55" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D55">
         <v>14</v>
@@ -2156,28 +2245,28 @@
       <c r="E55">
         <v>8</v>
       </c>
-      <c r="F55" s="7">
+      <c r="F55">
         <v>8</v>
       </c>
-      <c r="G55" s="10">
-        <v>0</v>
-      </c>
-      <c r="H55" s="8">
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55" s="7">
         <v>46179</v>
       </c>
       <c r="I55" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>21</v>
-      </c>
-      <c r="B56" s="8">
+        <v>24</v>
+      </c>
+      <c r="B56" s="7">
         <v>46181</v>
       </c>
       <c r="C56" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D56">
         <v>5</v>
@@ -2185,25 +2274,25 @@
       <c r="E56">
         <v>96</v>
       </c>
-      <c r="F56" s="7">
+      <c r="F56">
         <v>96</v>
       </c>
-      <c r="G56" s="10">
-        <v>0</v>
-      </c>
-      <c r="H56" s="8">
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>21</v>
-      </c>
-      <c r="B57" s="8">
+        <v>24</v>
+      </c>
+      <c r="B57" s="7">
         <v>46181</v>
       </c>
       <c r="C57" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="D57">
         <v>13</v>
@@ -2211,28 +2300,28 @@
       <c r="E57">
         <v>34</v>
       </c>
-      <c r="F57" s="7">
+      <c r="F57">
         <v>34</v>
       </c>
-      <c r="G57" s="10">
-        <v>0</v>
-      </c>
-      <c r="H57" s="8">
+      <c r="G57">
+        <v>0</v>
+      </c>
+      <c r="H57" s="7">
         <v>46179</v>
       </c>
       <c r="I57" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>21</v>
-      </c>
-      <c r="B58" s="8">
+        <v>24</v>
+      </c>
+      <c r="B58" s="7">
         <v>46181</v>
       </c>
       <c r="C58" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="D58">
         <v>1</v>
@@ -2240,25 +2329,25 @@
       <c r="E58">
         <v>55</v>
       </c>
-      <c r="F58" s="7">
+      <c r="F58">
         <v>55</v>
       </c>
-      <c r="G58" s="10">
-        <v>0</v>
-      </c>
-      <c r="H58" s="8">
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>21</v>
-      </c>
-      <c r="B59" s="8">
+        <v>24</v>
+      </c>
+      <c r="B59" s="7">
         <v>46181</v>
       </c>
       <c r="C59" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D59">
         <v>5</v>
@@ -2266,25 +2355,28 @@
       <c r="E59">
         <v>50</v>
       </c>
-      <c r="F59" s="7">
+      <c r="F59">
         <v>50</v>
       </c>
-      <c r="G59" s="10">
-        <v>0</v>
-      </c>
-      <c r="H59" s="8">
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59" s="7">
         <v>46179</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I59" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>21</v>
-      </c>
-      <c r="B60" s="8">
+        <v>24</v>
+      </c>
+      <c r="B60" s="7">
         <v>46181</v>
       </c>
       <c r="C60" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="D60">
         <v>9</v>
@@ -2292,28 +2384,28 @@
       <c r="E60">
         <v>52</v>
       </c>
-      <c r="F60" s="7">
+      <c r="F60">
         <v>0</v>
       </c>
       <c r="G60">
         <v>52</v>
       </c>
-      <c r="H60" s="8">
+      <c r="H60" s="7">
         <v>46179</v>
       </c>
       <c r="I60" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>21</v>
-      </c>
-      <c r="B61" s="8">
+        <v>24</v>
+      </c>
+      <c r="B61" s="7">
         <v>46181</v>
       </c>
       <c r="C61" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D61">
         <v>3</v>
@@ -2321,51 +2413,51 @@
       <c r="E61">
         <v>61</v>
       </c>
-      <c r="F61" s="7">
+      <c r="F61">
         <v>61</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
-      <c r="H61" s="8">
+      <c r="H61" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>21</v>
-      </c>
-      <c r="B62" s="8">
+        <v>24</v>
+      </c>
+      <c r="B62" s="7">
         <v>46181</v>
       </c>
       <c r="C62" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="D62" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E62">
         <v>107</v>
       </c>
-      <c r="F62" s="7">
+      <c r="F62">
         <v>107</v>
       </c>
-      <c r="G62" s="10">
-        <v>0</v>
-      </c>
-      <c r="H62" s="8">
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>21</v>
-      </c>
-      <c r="B63" s="8">
+        <v>24</v>
+      </c>
+      <c r="B63" s="7">
         <v>46181</v>
       </c>
       <c r="C63" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D63">
         <v>10</v>
@@ -2373,25 +2465,25 @@
       <c r="E63">
         <v>100</v>
       </c>
-      <c r="F63" s="7">
+      <c r="F63">
         <v>100</v>
       </c>
-      <c r="G63" s="10">
-        <v>0</v>
-      </c>
-      <c r="H63" s="8">
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>21</v>
-      </c>
-      <c r="B64" s="8">
+        <v>24</v>
+      </c>
+      <c r="B64" s="7">
         <v>46181</v>
       </c>
       <c r="C64" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="D64">
         <v>5</v>
@@ -2399,25 +2491,25 @@
       <c r="E64">
         <v>95</v>
       </c>
-      <c r="F64" s="7">
+      <c r="F64">
         <v>95</v>
       </c>
-      <c r="G64" s="10">
-        <v>0</v>
-      </c>
-      <c r="H64" s="8">
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>21</v>
-      </c>
-      <c r="B65" s="8">
+        <v>24</v>
+      </c>
+      <c r="B65" s="7">
         <v>46181</v>
       </c>
       <c r="C65" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D65">
         <v>7</v>
@@ -2425,25 +2517,25 @@
       <c r="E65">
         <v>44</v>
       </c>
-      <c r="F65" s="7">
+      <c r="F65">
         <v>44</v>
       </c>
-      <c r="G65" s="10">
-        <v>0</v>
-      </c>
-      <c r="H65" s="8">
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65" s="7">
         <v>46179</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>21</v>
-      </c>
-      <c r="B66" s="8">
+        <v>24</v>
+      </c>
+      <c r="B66" s="7">
         <v>46181</v>
       </c>
       <c r="C66" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="D66">
         <v>10</v>
@@ -2451,28 +2543,28 @@
       <c r="E66">
         <v>33</v>
       </c>
-      <c r="F66" s="7">
+      <c r="F66">
         <v>33</v>
       </c>
-      <c r="G66" s="10">
-        <v>0</v>
-      </c>
-      <c r="H66" s="8">
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66" s="7">
         <v>46179</v>
       </c>
       <c r="I66" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>21</v>
-      </c>
-      <c r="B67" s="8">
+        <v>24</v>
+      </c>
+      <c r="B67" s="7">
         <v>46181</v>
       </c>
       <c r="C67" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="D67">
         <v>6</v>
@@ -2480,29 +2572,29 @@
       <c r="E67">
         <v>33</v>
       </c>
-      <c r="F67" s="7">
+      <c r="F67">
         <v>33</v>
       </c>
-      <c r="G67" s="10">
-        <v>0</v>
-      </c>
-      <c r="H67" s="8">
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67" s="7">
         <v>46179</v>
       </c>
-      <c r="J67" s="9">
+      <c r="J67" s="8">
         <f>SUM(E36:E67)</f>
-        <v>2367</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A68" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B68" s="8">
+        <v>2167</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>24</v>
+      </c>
+      <c r="B68" s="7">
         <v>46185</v>
       </c>
       <c r="C68" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D68">
         <v>3</v>
@@ -2510,25 +2602,25 @@
       <c r="E68">
         <v>43</v>
       </c>
-      <c r="F68" s="7">
+      <c r="F68">
         <v>43</v>
       </c>
-      <c r="G68" s="10">
-        <v>0</v>
-      </c>
-      <c r="H68" s="8">
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68" s="7">
         <v>46183</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A69" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B69" s="8">
+    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>24</v>
+      </c>
+      <c r="B69" s="7">
         <v>46186</v>
       </c>
       <c r="C69" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D69">
         <v>12</v>
@@ -2536,25 +2628,25 @@
       <c r="E69">
         <v>177</v>
       </c>
-      <c r="F69" s="7">
+      <c r="F69">
         <v>177</v>
       </c>
-      <c r="G69" s="10">
-        <v>0</v>
-      </c>
-      <c r="H69" s="8">
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69" s="7">
         <v>46183</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A70" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B70" s="8">
+    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>24</v>
+      </c>
+      <c r="B70" s="7">
         <v>46187</v>
       </c>
       <c r="C70" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="D70">
         <v>10</v>
@@ -2562,25 +2654,25 @@
       <c r="E70">
         <v>79</v>
       </c>
-      <c r="F70" s="7">
+      <c r="F70">
         <v>79</v>
       </c>
-      <c r="G70" s="10">
-        <v>0</v>
-      </c>
-      <c r="H70" s="8">
+      <c r="G70">
+        <v>0</v>
+      </c>
+      <c r="H70" s="7">
         <v>46183</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A71" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B71" s="8">
+    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>24</v>
+      </c>
+      <c r="B71" s="7">
         <v>46188</v>
       </c>
       <c r="C71" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D71">
         <v>16</v>
@@ -2588,25 +2680,25 @@
       <c r="E71">
         <v>72</v>
       </c>
-      <c r="F71" s="7">
+      <c r="F71">
         <v>72</v>
       </c>
-      <c r="G71" s="10">
-        <v>0</v>
-      </c>
-      <c r="H71" s="8">
+      <c r="G71">
+        <v>0</v>
+      </c>
+      <c r="H71" s="7">
         <v>46183</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A72" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B72" s="8">
+    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>24</v>
+      </c>
+      <c r="B72" s="7">
         <v>46189</v>
       </c>
       <c r="C72" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="D72">
         <v>7</v>
@@ -2614,28 +2706,28 @@
       <c r="E72">
         <v>129</v>
       </c>
-      <c r="F72" s="7">
+      <c r="F72">
         <v>129</v>
       </c>
-      <c r="G72" s="10">
-        <v>0</v>
-      </c>
-      <c r="H72" s="8">
+      <c r="G72">
+        <v>0</v>
+      </c>
+      <c r="H72" s="7">
         <v>46183</v>
       </c>
-      <c r="I72" s="11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A73" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B73" s="8">
+      <c r="I72" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>24</v>
+      </c>
+      <c r="B73" s="7">
         <v>46190</v>
       </c>
       <c r="C73" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="D73">
         <v>11</v>
@@ -2643,28 +2735,28 @@
       <c r="E73">
         <v>120</v>
       </c>
-      <c r="F73" s="7">
+      <c r="F73">
         <v>120</v>
       </c>
-      <c r="G73" s="10">
-        <v>0</v>
-      </c>
-      <c r="H73" s="8">
+      <c r="G73">
+        <v>0</v>
+      </c>
+      <c r="H73" s="7">
         <v>46183</v>
       </c>
-      <c r="I73" s="11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A74" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B74" s="8">
+      <c r="I73" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>24</v>
+      </c>
+      <c r="B74" s="7">
         <v>46191</v>
       </c>
       <c r="C74" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D74">
         <v>8</v>
@@ -2672,28 +2764,28 @@
       <c r="E74">
         <v>61</v>
       </c>
-      <c r="F74" s="7">
+      <c r="F74">
         <v>61</v>
       </c>
-      <c r="G74" s="10">
-        <v>0</v>
-      </c>
-      <c r="H74" s="8">
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74" s="7">
         <v>46183</v>
       </c>
       <c r="I74" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A75" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B75" s="8">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>24</v>
+      </c>
+      <c r="B75" s="7">
         <v>46192</v>
       </c>
       <c r="C75" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="D75">
         <v>12</v>
@@ -2701,25 +2793,25 @@
       <c r="E75">
         <v>59</v>
       </c>
-      <c r="F75" s="7">
+      <c r="F75">
         <v>59</v>
       </c>
-      <c r="G75" s="10">
-        <v>0</v>
-      </c>
-      <c r="H75" s="8">
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75" s="7">
         <v>46183</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A76" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B76" s="8">
+    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>24</v>
+      </c>
+      <c r="B76" s="7">
         <v>46193</v>
       </c>
       <c r="C76" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D76">
         <v>4</v>
@@ -2727,28 +2819,28 @@
       <c r="E76">
         <v>100</v>
       </c>
-      <c r="F76" s="7">
+      <c r="F76">
         <v>100</v>
       </c>
-      <c r="G76" s="10">
-        <v>0</v>
-      </c>
-      <c r="H76" s="8">
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76" s="7">
         <v>46183</v>
       </c>
       <c r="I76" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A77" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B77" s="8">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>24</v>
+      </c>
+      <c r="B77" s="7">
         <v>46194</v>
       </c>
       <c r="C77" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="D77">
         <v>9</v>
@@ -2756,28 +2848,28 @@
       <c r="E77">
         <v>86</v>
       </c>
-      <c r="F77" s="7">
+      <c r="F77">
         <v>86</v>
       </c>
       <c r="G77">
         <v>0</v>
       </c>
-      <c r="H77" s="8">
+      <c r="H77" s="7">
         <v>46183</v>
       </c>
       <c r="I77" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A78" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B78" s="8">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>24</v>
+      </c>
+      <c r="B78" s="7">
         <v>46195</v>
       </c>
       <c r="C78" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D78">
         <v>39</v>
@@ -2785,28 +2877,28 @@
       <c r="E78">
         <v>113</v>
       </c>
-      <c r="F78" s="7">
+      <c r="F78">
         <v>0</v>
       </c>
       <c r="G78">
         <v>113</v>
       </c>
-      <c r="H78" s="8">
+      <c r="H78" s="7">
         <v>46183</v>
       </c>
       <c r="I78" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A79" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B79" s="8">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>24</v>
+      </c>
+      <c r="B79" s="7">
         <v>46196</v>
       </c>
       <c r="C79" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="D79">
         <v>15</v>
@@ -2814,25 +2906,25 @@
       <c r="E79">
         <v>32</v>
       </c>
-      <c r="F79" s="7">
+      <c r="F79">
         <v>32</v>
       </c>
       <c r="G79">
         <v>0</v>
       </c>
-      <c r="H79" s="8">
+      <c r="H79" s="7">
         <v>46183</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A80" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B80" s="8">
+    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>24</v>
+      </c>
+      <c r="B80" s="7">
         <v>46197</v>
       </c>
       <c r="C80" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D80">
         <v>14</v>
@@ -2840,24 +2932,54 @@
       <c r="E80">
         <v>0</v>
       </c>
-      <c r="F80" s="7">
+      <c r="F80">
         <v>0</v>
       </c>
       <c r="G80">
         <v>0</v>
       </c>
-      <c r="H80" s="8">
+      <c r="H80" s="7">
         <v>46183</v>
       </c>
       <c r="I80" t="s">
-        <v>44</v>
-      </c>
-      <c r="J80" s="9">
+        <v>38</v>
+      </c>
+      <c r="J80" s="8">
         <f>SUM(E68:E80)</f>
         <v>1071</v>
       </c>
     </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>24</v>
+      </c>
+      <c r="B81" s="7">
+        <v>46181</v>
+      </c>
+      <c r="C81" t="s">
+        <v>17</v>
+      </c>
+      <c r="D81">
+        <v>3</v>
+      </c>
+      <c r="E81">
+        <v>200</v>
+      </c>
+      <c r="F81">
+        <v>200</v>
+      </c>
+      <c r="J81" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A2:K80" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="A"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="3">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="A1:B1"/>
@@ -2869,92 +2991,102 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="1" max="1" width="20" style="9" customWidth="1"/>
+    <col min="2" max="2" width="16" style="9" customWidth="1"/>
+    <col min="3" max="4" width="8" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12" style="9" customWidth="1"/>
+    <col min="6" max="6" width="16" style="9" customWidth="1"/>
+    <col min="7" max="8" width="14" style="9" customWidth="1"/>
+    <col min="9" max="9" width="30" style="9" customWidth="1"/>
+    <col min="10" max="10" width="14" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="12" t="s">
+    <row r="1" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="15" t="s">
+      <c r="D1" s="14"/>
+      <c r="E1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J1" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I3" s="6"/>
+      <c r="J3" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2968,92 +3100,102 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="4" width="8" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="1" max="1" width="20" style="9" customWidth="1"/>
+    <col min="2" max="2" width="16" style="9" customWidth="1"/>
+    <col min="3" max="4" width="8" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12" style="9" customWidth="1"/>
+    <col min="6" max="6" width="16" style="9" customWidth="1"/>
+    <col min="7" max="8" width="14" style="9" customWidth="1"/>
+    <col min="9" max="9" width="30" style="9" customWidth="1"/>
+    <col min="10" max="10" width="14" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="12" t="s">
+    <row r="1" spans="1:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="13"/>
-      <c r="E1" s="15" t="s">
+      <c r="D1" s="14"/>
+      <c r="E1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J1" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I3" s="6"/>
+      <c r="J3" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>